<commit_message>
Corrige el modelo de Centralizadas y afina las alertas tras probar con 10 dependencias reales
- Centralizadas: la llave es el ID del registro (la actividad se repite); se cuentan actividades y registros
- Obligaciones sin avance: advertencia solo sin observación que lo explique y con cantidad programada
- Justificación del avance 0 en Análisis o Dificultades; se retira la regla que penalizaba usar Análisis
- Metas compartidas (PA vs PI): actividades de meta ajena y metas sin actividades dejan de ser errores
- Aviso en la matriz cuando la meta del export difiere de Drive; validaciones de Drive solo para las entidades cargadas
- Hallazgos con nombres legibles en pantalla y Excel; el indicador de alertas excluye lo informativo
- Documentación y preguntas abiertas actualizadas

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QxWYGkwBcmDdXSGawYPFsD
</commit_message>
<xml_diff>
--- a/data/ejemplos/ejemplo_Centralizadas.xlsx
+++ b/data/ejemplos/ejemplo_Centralizadas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF7"/>
+  <dimension ref="A1:AF8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1212,6 +1212,130 @@
         </is>
       </c>
       <c r="AF7" t="inlineStr">
+        <is>
+          <t>ACTIVO</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>12005</v>
+      </c>
+      <c r="B8" t="n">
+        <v>9999</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>SRIA DE EJEMPLO  DE LA INFORM</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>PI99-000002</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Proyecto de ejemplo dos</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>2024009990002</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>MP9900202029902002</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>ENTREGAR 10 DOCUMENTOS TÉCNICOS</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>9902002</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Servicio de ejemplo 9902002</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>990200200</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Personas atendidas 9902002</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>PI99-000002/1/1/01/01</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Contratar consultoría</t>
+        </is>
+      </c>
+      <c r="O8" t="n">
+        <v>121000</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Ingresos corrientes de Libre Destinación</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>100.000.000</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>100.000.000</t>
+        </is>
+      </c>
+      <c r="S8" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>100.000.000</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>SIN EJECUCION</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>Número</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>de personas</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>Número de personas</t>
+        </is>
+      </c>
+      <c r="AB8" t="n">
+        <v>4</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
         <is>
           <t>ACTIVO</t>
         </is>

</xml_diff>